<commit_message>
Data P01-P07 and new charts
</commit_message>
<xml_diff>
--- a/Output/merged_data.xlsx
+++ b/Output/merged_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EU23"/>
+  <dimension ref="A1:EI23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -781,405 +781,345 @@
       </c>
       <c r="BS1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_2</t>
+          <t>M1_SSI_3</t>
         </is>
       </c>
       <c r="BT1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_3</t>
+          <t>M1_SSI_9</t>
         </is>
       </c>
       <c r="BU1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_4</t>
+          <t>M1_SSI_10</t>
         </is>
       </c>
       <c r="BV1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_5</t>
+          <t>M1_adverse_events</t>
         </is>
       </c>
       <c r="BW1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_6</t>
+          <t>M1_total_score</t>
         </is>
       </c>
       <c r="BX1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_7</t>
+          <t>M1_competence_score</t>
         </is>
       </c>
       <c r="BY1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_8</t>
+          <t>M1_adaptability_score</t>
         </is>
       </c>
       <c r="BZ1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_9</t>
+          <t>M1_self_esteem_score</t>
         </is>
       </c>
       <c r="CA1" s="1" t="inlineStr">
         <is>
-          <t>M1_SSI_10</t>
+          <t>M2_1.1_score</t>
         </is>
       </c>
       <c r="CB1" s="1" t="inlineStr">
         <is>
-          <t>M1_adverse_events</t>
+          <t>M2_1.1_time</t>
         </is>
       </c>
       <c r="CC1" s="1" t="inlineStr">
         <is>
-          <t>M1_total_score</t>
+          <t>M2_1.2_score</t>
         </is>
       </c>
       <c r="CD1" s="1" t="inlineStr">
         <is>
-          <t>M1_competence_score</t>
+          <t>M2_1.2_time</t>
         </is>
       </c>
       <c r="CE1" s="1" t="inlineStr">
         <is>
-          <t>M1_adaptability_score</t>
+          <t>M2_1.3_score</t>
         </is>
       </c>
       <c r="CF1" s="1" t="inlineStr">
         <is>
-          <t>M1_self_esteem_score</t>
+          <t>M2_1.3_time</t>
         </is>
       </c>
       <c r="CG1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.1_score</t>
+          <t>M2_1.4</t>
         </is>
       </c>
       <c r="CH1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.1_time</t>
+          <t>M2_1.5</t>
         </is>
       </c>
       <c r="CI1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.2_score</t>
+          <t>M2_2.1_score</t>
         </is>
       </c>
       <c r="CJ1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.2_time</t>
+          <t>M2_2.1_time</t>
         </is>
       </c>
       <c r="CK1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.3_score</t>
+          <t>M2_2.2_score</t>
         </is>
       </c>
       <c r="CL1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.3_time</t>
+          <t>M2_2.2_time</t>
         </is>
       </c>
       <c r="CM1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.4</t>
+          <t>M2_2.3_score</t>
         </is>
       </c>
       <c r="CN1" s="1" t="inlineStr">
         <is>
-          <t>M2_1.5</t>
+          <t>M2_2.3_time</t>
         </is>
       </c>
       <c r="CO1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.1_score</t>
+          <t>M2_2.4_score</t>
         </is>
       </c>
       <c r="CP1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.1_time</t>
+          <t>M2_2.4_time</t>
         </is>
       </c>
       <c r="CQ1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.2_score</t>
+          <t>M2_2.5</t>
         </is>
       </c>
       <c r="CR1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.2_time</t>
+          <t>M2_2.6</t>
         </is>
       </c>
       <c r="CS1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.3_score</t>
+          <t>M2_3.1_score</t>
         </is>
       </c>
       <c r="CT1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.3_time</t>
+          <t>M2_3.1_time</t>
         </is>
       </c>
       <c r="CU1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.4_score</t>
+          <t>M2_3.2_score</t>
         </is>
       </c>
       <c r="CV1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.4_time</t>
+          <t>M2_3.2_time</t>
         </is>
       </c>
       <c r="CW1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.5</t>
+          <t>M2_3.3_score</t>
         </is>
       </c>
       <c r="CX1" s="1" t="inlineStr">
         <is>
-          <t>M2_2.6</t>
+          <t>M2_3.3_time</t>
         </is>
       </c>
       <c r="CY1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.1_score</t>
+          <t>M2_3.4_score</t>
         </is>
       </c>
       <c r="CZ1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.1_time</t>
+          <t>M2_3.4_time</t>
         </is>
       </c>
       <c r="DA1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.2_score</t>
+          <t>M2_3.5_score</t>
         </is>
       </c>
       <c r="DB1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.2_time</t>
+          <t>M2_3.5_time</t>
         </is>
       </c>
       <c r="DC1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.3_score</t>
+          <t>M2_3.6</t>
         </is>
       </c>
       <c r="DD1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.3_time</t>
+          <t>M2_3.7</t>
         </is>
       </c>
       <c r="DE1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.4_score</t>
+          <t>M2_4.1_score</t>
         </is>
       </c>
       <c r="DF1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.4_time</t>
+          <t>M2_4.1_time</t>
         </is>
       </c>
       <c r="DG1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.5_score</t>
+          <t>M2_4.2_score</t>
         </is>
       </c>
       <c r="DH1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.5_time</t>
+          <t>M2_4.2_time</t>
         </is>
       </c>
       <c r="DI1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.6</t>
+          <t>M2_4.3_score</t>
         </is>
       </c>
       <c r="DJ1" s="1" t="inlineStr">
         <is>
-          <t>M2_3.7</t>
+          <t>M2_4.3_time</t>
         </is>
       </c>
       <c r="DK1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.1_score</t>
+          <t>M2_4.4_score</t>
         </is>
       </c>
       <c r="DL1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.1_time</t>
+          <t>M2_4.4_time</t>
         </is>
       </c>
       <c r="DM1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.2_score</t>
+          <t>M2_4.5</t>
         </is>
       </c>
       <c r="DN1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.2_time</t>
+          <t>M2_4.6</t>
         </is>
       </c>
       <c r="DO1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.3_score</t>
+          <t>M2_5.1_score</t>
         </is>
       </c>
       <c r="DP1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.3_time</t>
+          <t>M2_5.1_time</t>
         </is>
       </c>
       <c r="DQ1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.4_score</t>
+          <t>M2_5.2_score</t>
         </is>
       </c>
       <c r="DR1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.4_time</t>
+          <t>M2_5.2_time</t>
         </is>
       </c>
       <c r="DS1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.5</t>
+          <t>M2_5.3</t>
         </is>
       </c>
       <c r="DT1" s="1" t="inlineStr">
         <is>
-          <t>M2_4.6</t>
+          <t>M2_5.4</t>
         </is>
       </c>
       <c r="DU1" s="1" t="inlineStr">
         <is>
-          <t>M2_5.1_score</t>
+          <t>M2_6.1_score</t>
         </is>
       </c>
       <c r="DV1" s="1" t="inlineStr">
         <is>
-          <t>M2_5.1_time</t>
+          <t>M2_6.1_time</t>
         </is>
       </c>
       <c r="DW1" s="1" t="inlineStr">
         <is>
-          <t>M2_5.2_score</t>
+          <t>M2_6.2_score</t>
         </is>
       </c>
       <c r="DX1" s="1" t="inlineStr">
         <is>
-          <t>M2_5.2_time</t>
+          <t>M2_6.2_time</t>
         </is>
       </c>
       <c r="DY1" s="1" t="inlineStr">
         <is>
-          <t>M2_5.3</t>
+          <t>M2_6.3</t>
         </is>
       </c>
       <c r="DZ1" s="1" t="inlineStr">
         <is>
-          <t>M2_5.4</t>
+          <t>M2_6.4</t>
         </is>
       </c>
       <c r="EA1" s="1" t="inlineStr">
         <is>
-          <t>M2_6.1_score</t>
+          <t>M2_SSI_1</t>
         </is>
       </c>
       <c r="EB1" s="1" t="inlineStr">
         <is>
-          <t>M2_6.1_time</t>
+          <t>M2_SSI_3</t>
         </is>
       </c>
       <c r="EC1" s="1" t="inlineStr">
         <is>
-          <t>M2_6.2_score</t>
+          <t>M2_SSI_9</t>
         </is>
       </c>
       <c r="ED1" s="1" t="inlineStr">
         <is>
-          <t>M2_6.2_time</t>
+          <t>M2_SSI_10</t>
         </is>
       </c>
       <c r="EE1" s="1" t="inlineStr">
         <is>
-          <t>M2_6.3</t>
+          <t>M2_adverse_events</t>
         </is>
       </c>
       <c r="EF1" s="1" t="inlineStr">
         <is>
-          <t>M2_6.4</t>
+          <t>M2_total_score</t>
         </is>
       </c>
       <c r="EG1" s="1" t="inlineStr">
         <is>
-          <t>M2_SSI_1</t>
+          <t>M2_competence_score</t>
         </is>
       </c>
       <c r="EH1" s="1" t="inlineStr">
         <is>
-          <t>M2_SSI_2</t>
+          <t>M2_adaptability_score</t>
         </is>
       </c>
       <c r="EI1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_3</t>
-        </is>
-      </c>
-      <c r="EJ1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_4</t>
-        </is>
-      </c>
-      <c r="EK1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_5</t>
-        </is>
-      </c>
-      <c r="EL1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_6</t>
-        </is>
-      </c>
-      <c r="EM1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_7</t>
-        </is>
-      </c>
-      <c r="EN1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_8</t>
-        </is>
-      </c>
-      <c r="EO1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_9</t>
-        </is>
-      </c>
-      <c r="EP1" s="1" t="inlineStr">
-        <is>
-          <t>M2_SSI_10</t>
-        </is>
-      </c>
-      <c r="EQ1" s="1" t="inlineStr">
-        <is>
-          <t>M2_adverse_events</t>
-        </is>
-      </c>
-      <c r="ER1" s="1" t="inlineStr">
-        <is>
-          <t>M2_total_score</t>
-        </is>
-      </c>
-      <c r="ES1" s="1" t="inlineStr">
-        <is>
-          <t>M2_competence_score</t>
-        </is>
-      </c>
-      <c r="ET1" s="1" t="inlineStr">
-        <is>
-          <t>M2_adaptability_score</t>
-        </is>
-      </c>
-      <c r="EU1" s="1" t="inlineStr">
         <is>
           <t>M2_self_esteem_score</t>
         </is>
@@ -1231,8 +1171,10 @@
           <t>82kg</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>1</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="K2" t="n">
         <v>1</v>
@@ -1251,8 +1193,10 @@
         <v>30</v>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="n">
-        <v>8</v>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
@@ -1386,137 +1330,145 @@
       <c r="BR2" t="n">
         <v>7</v>
       </c>
-      <c r="BS2" t="inlineStr"/>
+      <c r="BS2" t="n">
+        <v>6</v>
+      </c>
       <c r="BT2" t="n">
         <v>6</v>
       </c>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr"/>
-      <c r="BW2" t="inlineStr"/>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
+      <c r="BU2" t="n">
+        <v>6</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>1.423</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>2</v>
+      </c>
       <c r="BZ2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>55</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>26</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>15</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>7</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>7</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>20</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>21</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>8</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>40</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>5</v>
+      </c>
+      <c r="CR2" t="n">
         <v>6</v>
       </c>
-      <c r="CA2" t="n">
-        <v>6</v>
-      </c>
-      <c r="CB2" t="n">
+      <c r="CS2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>58</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>32</v>
+      </c>
+      <c r="CW2" t="n">
+        <v>3</v>
+      </c>
+      <c r="CX2" t="n">
+        <v>86</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CZ2" t="n">
+        <v>147</v>
+      </c>
+      <c r="DA2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB2" t="n">
+        <v>104</v>
+      </c>
+      <c r="DC2" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD2" t="n">
+        <v>5</v>
+      </c>
+      <c r="DE2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF2" t="n">
+        <v>10</v>
+      </c>
+      <c r="DG2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DH2" t="n">
+        <v>10</v>
+      </c>
+      <c r="DI2" t="n">
         <v>0</v>
       </c>
-      <c r="CC2" t="n">
-        <v>1.423</v>
-      </c>
-      <c r="CD2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="CE2" t="n">
-        <v>2</v>
-      </c>
-      <c r="CF2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="CG2" t="n">
-        <v>3</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>55</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>26</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>3</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>15</v>
-      </c>
-      <c r="CM2" t="n">
-        <v>7</v>
-      </c>
-      <c r="CN2" t="n">
-        <v>7</v>
-      </c>
-      <c r="CO2" t="n">
-        <v>2</v>
-      </c>
-      <c r="CP2" t="n">
-        <v>20</v>
-      </c>
-      <c r="CQ2" t="n">
-        <v>3</v>
-      </c>
-      <c r="CR2" t="n">
-        <v>21</v>
-      </c>
-      <c r="CS2" t="n">
-        <v>3</v>
-      </c>
-      <c r="CT2" t="n">
-        <v>8</v>
-      </c>
-      <c r="CU2" t="n">
-        <v>2</v>
-      </c>
-      <c r="CV2" t="n">
-        <v>40</v>
-      </c>
-      <c r="CW2" t="n">
-        <v>5</v>
-      </c>
-      <c r="CX2" t="n">
-        <v>6</v>
-      </c>
-      <c r="CY2" t="n">
-        <v>3</v>
-      </c>
-      <c r="CZ2" t="n">
-        <v>58</v>
-      </c>
-      <c r="DA2" t="n">
-        <v>3</v>
-      </c>
-      <c r="DB2" t="n">
-        <v>32</v>
-      </c>
-      <c r="DC2" t="n">
-        <v>3</v>
-      </c>
-      <c r="DD2" t="n">
-        <v>86</v>
-      </c>
-      <c r="DE2" t="n">
-        <v>2</v>
-      </c>
-      <c r="DF2" t="n">
-        <v>147</v>
-      </c>
-      <c r="DG2" t="n">
-        <v>3</v>
-      </c>
-      <c r="DH2" t="n">
-        <v>104</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>5</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>5</v>
-      </c>
+      <c r="DJ2" t="inlineStr"/>
       <c r="DK2" t="n">
-        <v>3</v>
-      </c>
-      <c r="DL2" t="n">
-        <v>10</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="DL2" t="inlineStr"/>
       <c r="DM2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="DN2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="DO2" t="n">
         <v>0</v>
@@ -1526,12 +1478,8 @@
         <v>0</v>
       </c>
       <c r="DR2" t="inlineStr"/>
-      <c r="DS2" t="n">
-        <v>7</v>
-      </c>
-      <c r="DT2" t="n">
-        <v>7</v>
-      </c>
+      <c r="DS2" t="inlineStr"/>
+      <c r="DT2" t="inlineStr"/>
       <c r="DU2" t="n">
         <v>0</v>
       </c>
@@ -1543,46 +1491,30 @@
       <c r="DY2" t="inlineStr"/>
       <c r="DZ2" t="inlineStr"/>
       <c r="EA2" t="n">
+        <v>7</v>
+      </c>
+      <c r="EB2" t="n">
+        <v>6</v>
+      </c>
+      <c r="EC2" t="n">
+        <v>6</v>
+      </c>
+      <c r="ED2" t="n">
+        <v>7</v>
+      </c>
+      <c r="EE2" t="n">
         <v>0</v>
       </c>
-      <c r="EB2" t="inlineStr"/>
-      <c r="EC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="ED2" t="inlineStr"/>
-      <c r="EE2" t="inlineStr"/>
-      <c r="EF2" t="inlineStr"/>
+      <c r="EF2" t="n">
+        <v>1.577</v>
+      </c>
       <c r="EG2" t="n">
-        <v>7</v>
-      </c>
-      <c r="EH2" t="inlineStr"/>
+        <v>1.167</v>
+      </c>
+      <c r="EH2" t="n">
+        <v>1.667</v>
+      </c>
       <c r="EI2" t="n">
-        <v>6</v>
-      </c>
-      <c r="EJ2" t="inlineStr"/>
-      <c r="EK2" t="inlineStr"/>
-      <c r="EL2" t="inlineStr"/>
-      <c r="EM2" t="inlineStr"/>
-      <c r="EN2" t="inlineStr"/>
-      <c r="EO2" t="n">
-        <v>6</v>
-      </c>
-      <c r="EP2" t="n">
-        <v>7</v>
-      </c>
-      <c r="EQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="ER2" t="n">
-        <v>1.577</v>
-      </c>
-      <c r="ES2" t="n">
-        <v>1.167</v>
-      </c>
-      <c r="ET2" t="n">
-        <v>1.667</v>
-      </c>
-      <c r="EU2" t="n">
         <v>2.125</v>
       </c>
     </row>
@@ -1632,8 +1564,10 @@
           <t>117kg</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>0</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="K3" t="n">
         <v>2</v>
@@ -1653,15 +1587,21 @@
       <c r="R3" t="n">
         <v>3</v>
       </c>
-      <c r="S3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>37</v>
+      </c>
       <c r="T3" t="n">
         <v>3</v>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>27</v>
+      </c>
       <c r="V3" t="n">
         <v>3</v>
       </c>
-      <c r="W3" t="inlineStr"/>
+      <c r="W3" t="n">
+        <v>25</v>
+      </c>
       <c r="X3" t="n">
         <v>5</v>
       </c>
@@ -1671,19 +1611,27 @@
       <c r="Z3" t="n">
         <v>3</v>
       </c>
-      <c r="AA3" t="inlineStr"/>
+      <c r="AA3" t="n">
+        <v>40</v>
+      </c>
       <c r="AB3" t="n">
         <v>3</v>
       </c>
-      <c r="AC3" t="inlineStr"/>
+      <c r="AC3" t="n">
+        <v>27</v>
+      </c>
       <c r="AD3" t="n">
         <v>3</v>
       </c>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AE3" t="n">
+        <v>18</v>
+      </c>
       <c r="AF3" t="n">
         <v>3</v>
       </c>
-      <c r="AG3" t="inlineStr"/>
+      <c r="AG3" t="n">
+        <v>55</v>
+      </c>
       <c r="AH3" t="n">
         <v>5</v>
       </c>
@@ -1693,23 +1641,33 @@
       <c r="AJ3" t="n">
         <v>3</v>
       </c>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AK3" t="n">
+        <v>63</v>
+      </c>
       <c r="AL3" t="n">
         <v>3</v>
       </c>
-      <c r="AM3" t="inlineStr"/>
+      <c r="AM3" t="n">
+        <v>60</v>
+      </c>
       <c r="AN3" t="n">
         <v>3</v>
       </c>
-      <c r="AO3" t="inlineStr"/>
+      <c r="AO3" t="n">
+        <v>50</v>
+      </c>
       <c r="AP3" t="n">
         <v>3</v>
       </c>
-      <c r="AQ3" t="inlineStr"/>
+      <c r="AQ3" t="n">
+        <v>40</v>
+      </c>
       <c r="AR3" t="n">
         <v>2</v>
       </c>
-      <c r="AS3" t="inlineStr"/>
+      <c r="AS3" t="n">
+        <v>91</v>
+      </c>
       <c r="AT3" t="n">
         <v>5</v>
       </c>
@@ -1719,11 +1677,15 @@
       <c r="AV3" t="n">
         <v>3</v>
       </c>
-      <c r="AW3" t="inlineStr"/>
+      <c r="AW3" t="n">
+        <v>10</v>
+      </c>
       <c r="AX3" t="n">
         <v>3</v>
       </c>
-      <c r="AY3" t="inlineStr"/>
+      <c r="AY3" t="n">
+        <v>13</v>
+      </c>
       <c r="AZ3" t="n">
         <v>0</v>
       </c>
@@ -1761,183 +1723,211 @@
       <c r="BR3" t="n">
         <v>4</v>
       </c>
-      <c r="BS3" t="inlineStr"/>
+      <c r="BS3" t="n">
+        <v>5</v>
+      </c>
       <c r="BT3" t="n">
+        <v>6</v>
+      </c>
+      <c r="BU3" t="n">
         <v>5</v>
       </c>
-      <c r="BU3" t="inlineStr"/>
-      <c r="BV3" t="inlineStr"/>
-      <c r="BW3" t="inlineStr"/>
-      <c r="BX3" t="inlineStr"/>
-      <c r="BY3" t="inlineStr"/>
+      <c r="BV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>2.167</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>2.5</v>
+      </c>
       <c r="BZ3" t="n">
+        <v>1.375</v>
+      </c>
+      <c r="CA3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB3" t="n">
+        <v>30</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD3" t="n">
+        <v>20</v>
+      </c>
+      <c r="CE3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF3" t="n">
+        <v>22</v>
+      </c>
+      <c r="CG3" t="n">
         <v>6</v>
       </c>
-      <c r="CA3" t="n">
+      <c r="CH3" t="n">
+        <v>7</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>21</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>17</v>
+      </c>
+      <c r="CM3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CN3" t="n">
+        <v>10</v>
+      </c>
+      <c r="CO3" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP3" t="n">
+        <v>22</v>
+      </c>
+      <c r="CQ3" t="n">
         <v>5</v>
       </c>
-      <c r="CB3" t="n">
+      <c r="CR3" t="n">
+        <v>7</v>
+      </c>
+      <c r="CS3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CT3" t="n">
+        <v>68</v>
+      </c>
+      <c r="CU3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CV3" t="n">
+        <v>83</v>
+      </c>
+      <c r="CW3" t="n">
+        <v>3</v>
+      </c>
+      <c r="CX3" t="n">
+        <v>100</v>
+      </c>
+      <c r="CY3" t="n">
+        <v>2</v>
+      </c>
+      <c r="CZ3" t="n">
+        <v>140</v>
+      </c>
+      <c r="DA3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB3" t="n">
+        <v>135</v>
+      </c>
+      <c r="DC3" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD3" t="n">
+        <v>5</v>
+      </c>
+      <c r="DE3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF3" t="n">
+        <v>6</v>
+      </c>
+      <c r="DG3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DH3" t="n">
+        <v>9</v>
+      </c>
+      <c r="DI3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DJ3" t="n">
+        <v>95</v>
+      </c>
+      <c r="DK3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DL3" t="n">
+        <v>80</v>
+      </c>
+      <c r="DM3" t="n">
+        <v>5</v>
+      </c>
+      <c r="DN3" t="n">
+        <v>5</v>
+      </c>
+      <c r="DO3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DP3" t="n">
+        <v>77</v>
+      </c>
+      <c r="DQ3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DR3" t="n">
+        <v>45</v>
+      </c>
+      <c r="DS3" t="n">
+        <v>7</v>
+      </c>
+      <c r="DT3" t="n">
+        <v>6</v>
+      </c>
+      <c r="DU3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DV3" t="n">
+        <v>130</v>
+      </c>
+      <c r="DW3" t="n">
+        <v>3</v>
+      </c>
+      <c r="DX3" t="n">
+        <v>74</v>
+      </c>
+      <c r="DY3" t="n">
+        <v>7</v>
+      </c>
+      <c r="DZ3" t="n">
+        <v>7</v>
+      </c>
+      <c r="EA3" t="n">
+        <v>6</v>
+      </c>
+      <c r="EB3" t="n">
+        <v>7</v>
+      </c>
+      <c r="EC3" t="n">
+        <v>5</v>
+      </c>
+      <c r="ED3" t="n">
+        <v>7</v>
+      </c>
+      <c r="EE3" t="n">
         <v>0</v>
       </c>
-      <c r="CC3" t="n">
-        <v>2</v>
-      </c>
-      <c r="CD3" t="n">
-        <v>2.167</v>
-      </c>
-      <c r="CE3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="CF3" t="n">
-        <v>1.375</v>
-      </c>
-      <c r="CG3" t="n">
-        <v>3</v>
-      </c>
-      <c r="CH3" t="inlineStr"/>
-      <c r="CI3" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ3" t="inlineStr"/>
-      <c r="CK3" t="n">
-        <v>3</v>
-      </c>
-      <c r="CL3" t="inlineStr"/>
-      <c r="CM3" t="n">
-        <v>6</v>
-      </c>
-      <c r="CN3" t="n">
-        <v>7</v>
-      </c>
-      <c r="CO3" t="n">
-        <v>2</v>
-      </c>
-      <c r="CP3" t="inlineStr"/>
-      <c r="CQ3" t="n">
-        <v>3</v>
-      </c>
-      <c r="CR3" t="inlineStr"/>
-      <c r="CS3" t="n">
-        <v>3</v>
-      </c>
-      <c r="CT3" t="inlineStr"/>
-      <c r="CU3" t="n">
-        <v>2</v>
-      </c>
-      <c r="CV3" t="inlineStr"/>
-      <c r="CW3" t="n">
-        <v>5</v>
-      </c>
-      <c r="CX3" t="n">
-        <v>7</v>
-      </c>
-      <c r="CY3" t="n">
-        <v>3</v>
-      </c>
-      <c r="CZ3" t="inlineStr"/>
-      <c r="DA3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DB3" t="inlineStr"/>
-      <c r="DC3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DD3" t="inlineStr"/>
-      <c r="DE3" t="n">
-        <v>2</v>
-      </c>
-      <c r="DF3" t="inlineStr"/>
-      <c r="DG3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DH3" t="inlineStr"/>
-      <c r="DI3" t="n">
-        <v>5</v>
-      </c>
-      <c r="DJ3" t="n">
-        <v>5</v>
-      </c>
-      <c r="DK3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DL3" t="inlineStr"/>
-      <c r="DM3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DN3" t="inlineStr"/>
-      <c r="DO3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DP3" t="inlineStr"/>
-      <c r="DQ3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DR3" t="inlineStr"/>
-      <c r="DS3" t="n">
-        <v>5</v>
-      </c>
-      <c r="DT3" t="n">
-        <v>5</v>
-      </c>
-      <c r="DU3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DV3" t="inlineStr"/>
-      <c r="DW3" t="n">
-        <v>3</v>
-      </c>
-      <c r="DX3" t="inlineStr"/>
-      <c r="DY3" t="n">
-        <v>7</v>
-      </c>
-      <c r="DZ3" t="n">
-        <v>6</v>
-      </c>
-      <c r="EA3" t="n">
-        <v>3</v>
-      </c>
-      <c r="EB3" t="inlineStr"/>
-      <c r="EC3" t="n">
-        <v>3</v>
-      </c>
-      <c r="ED3" t="inlineStr"/>
-      <c r="EE3" t="n">
-        <v>7</v>
-      </c>
       <c r="EF3" t="n">
-        <v>7</v>
+        <v>2.846</v>
       </c>
       <c r="EG3" t="n">
-        <v>6</v>
-      </c>
-      <c r="EH3" t="inlineStr"/>
+        <v>2.75</v>
+      </c>
+      <c r="EH3" t="n">
+        <v>3</v>
+      </c>
       <c r="EI3" t="n">
-        <v>7</v>
-      </c>
-      <c r="EJ3" t="inlineStr"/>
-      <c r="EK3" t="inlineStr"/>
-      <c r="EL3" t="inlineStr"/>
-      <c r="EM3" t="inlineStr"/>
-      <c r="EN3" t="inlineStr"/>
-      <c r="EO3" t="n">
-        <v>5</v>
-      </c>
-      <c r="EP3" t="n">
-        <v>7</v>
-      </c>
-      <c r="EQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="ER3" t="n">
-        <v>2.846</v>
-      </c>
-      <c r="ES3" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="ET3" t="n">
-        <v>3</v>
-      </c>
-      <c r="EU3" t="n">
         <v>2.875</v>
       </c>
     </row>
@@ -1987,8 +1977,10 @@
           <t>78kg</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>1</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="K4" t="n">
         <v>1</v>
@@ -2007,22 +1999,30 @@
         <v>29</v>
       </c>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="n">
-        <v>7.5</v>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
         <v>3</v>
       </c>
-      <c r="S4" t="inlineStr"/>
+      <c r="S4" t="n">
+        <v>44</v>
+      </c>
       <c r="T4" t="n">
         <v>3</v>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>35</v>
+      </c>
       <c r="V4" t="n">
         <v>3</v>
       </c>
-      <c r="W4" t="inlineStr"/>
+      <c r="W4" t="n">
+        <v>15</v>
+      </c>
       <c r="X4" t="n">
         <v>7</v>
       </c>
@@ -2032,19 +2032,27 @@
       <c r="Z4" t="n">
         <v>3</v>
       </c>
-      <c r="AA4" t="inlineStr"/>
+      <c r="AA4" t="n">
+        <v>26</v>
+      </c>
       <c r="AB4" t="n">
         <v>3</v>
       </c>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AC4" t="n">
+        <v>17</v>
+      </c>
       <c r="AD4" t="n">
         <v>3</v>
       </c>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AE4" t="n">
+        <v>8</v>
+      </c>
       <c r="AF4" t="n">
         <v>2</v>
       </c>
-      <c r="AG4" t="inlineStr"/>
+      <c r="AG4" t="n">
+        <v>12</v>
+      </c>
       <c r="AH4" t="n">
         <v>5</v>
       </c>
@@ -2054,23 +2062,33 @@
       <c r="AJ4" t="n">
         <v>2</v>
       </c>
-      <c r="AK4" t="inlineStr"/>
+      <c r="AK4" t="n">
+        <v>85</v>
+      </c>
       <c r="AL4" t="n">
         <v>3</v>
       </c>
-      <c r="AM4" t="inlineStr"/>
+      <c r="AM4" t="n">
+        <v>26</v>
+      </c>
       <c r="AN4" t="n">
         <v>1</v>
       </c>
-      <c r="AO4" t="inlineStr"/>
+      <c r="AO4" t="n">
+        <v>245</v>
+      </c>
       <c r="AP4" t="n">
         <v>2</v>
       </c>
-      <c r="AQ4" t="inlineStr"/>
+      <c r="AQ4" t="n">
+        <v>88</v>
+      </c>
       <c r="AR4" t="n">
         <v>3</v>
       </c>
-      <c r="AS4" t="inlineStr"/>
+      <c r="AS4" t="n">
+        <v>83</v>
+      </c>
       <c r="AT4" t="n">
         <v>5</v>
       </c>
@@ -2080,11 +2098,15 @@
       <c r="AV4" t="n">
         <v>3</v>
       </c>
-      <c r="AW4" t="inlineStr"/>
+      <c r="AW4" t="n">
+        <v>10</v>
+      </c>
       <c r="AX4" t="n">
         <v>3</v>
       </c>
-      <c r="AY4" t="inlineStr"/>
+      <c r="AY4" t="n">
+        <v>8</v>
+      </c>
       <c r="AZ4" t="n">
         <v>0</v>
       </c>
@@ -2122,118 +2144,162 @@
       <c r="BR4" t="n">
         <v>7</v>
       </c>
-      <c r="BS4" t="inlineStr"/>
+      <c r="BS4" t="n">
+        <v>7</v>
+      </c>
       <c r="BT4" t="n">
         <v>7</v>
       </c>
-      <c r="BU4" t="inlineStr"/>
-      <c r="BV4" t="inlineStr"/>
-      <c r="BW4" t="inlineStr"/>
-      <c r="BX4" t="inlineStr"/>
-      <c r="BY4" t="inlineStr"/>
+      <c r="BU4" t="n">
+        <v>7</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>1.923</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>1.83</v>
+      </c>
       <c r="BZ4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="CA4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="CB4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="CC4" t="n">
-        <v>1.923</v>
+        <v>3</v>
       </c>
       <c r="CD4" t="n">
-        <v>1.91</v>
+        <v>16</v>
       </c>
       <c r="CE4" t="n">
-        <v>1.83</v>
+        <v>3</v>
       </c>
       <c r="CF4" t="n">
-        <v>1.86</v>
+        <v>44</v>
       </c>
       <c r="CG4" t="n">
-        <v>3</v>
-      </c>
-      <c r="CH4" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="CH4" t="n">
+        <v>7</v>
+      </c>
       <c r="CI4" t="n">
-        <v>3</v>
-      </c>
-      <c r="CJ4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>20</v>
+      </c>
       <c r="CK4" t="n">
         <v>3</v>
       </c>
-      <c r="CL4" t="inlineStr"/>
+      <c r="CL4" t="n">
+        <v>17</v>
+      </c>
       <c r="CM4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="CN4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="CO4" t="n">
-        <v>2</v>
-      </c>
-      <c r="CP4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="CP4" t="n">
+        <v>18</v>
+      </c>
       <c r="CQ4" t="n">
-        <v>3</v>
-      </c>
-      <c r="CR4" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="CR4" t="n">
+        <v>7</v>
+      </c>
       <c r="CS4" t="n">
         <v>3</v>
       </c>
-      <c r="CT4" t="inlineStr"/>
+      <c r="CT4" t="n">
+        <v>63</v>
+      </c>
       <c r="CU4" t="n">
         <v>3</v>
       </c>
-      <c r="CV4" t="inlineStr"/>
+      <c r="CV4" t="n">
+        <v>45</v>
+      </c>
       <c r="CW4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="CX4" t="n">
-        <v>7</v>
+        <v>244</v>
       </c>
       <c r="CY4" t="n">
-        <v>3</v>
-      </c>
-      <c r="CZ4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="CZ4" t="n">
+        <v>196</v>
+      </c>
       <c r="DA4" t="n">
         <v>3</v>
       </c>
-      <c r="DB4" t="inlineStr"/>
+      <c r="DB4" t="n">
+        <v>60</v>
+      </c>
       <c r="DC4" t="n">
-        <v>2</v>
-      </c>
-      <c r="DD4" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="DD4" t="n">
+        <v>7</v>
+      </c>
       <c r="DE4" t="n">
-        <v>2</v>
-      </c>
-      <c r="DF4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="DF4" t="n">
+        <v>8</v>
+      </c>
       <c r="DG4" t="n">
         <v>3</v>
       </c>
-      <c r="DH4" t="inlineStr"/>
+      <c r="DH4" t="n">
+        <v>9</v>
+      </c>
       <c r="DI4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="DJ4" t="n">
-        <v>7</v>
+        <v>210</v>
       </c>
       <c r="DK4" t="n">
         <v>3</v>
       </c>
-      <c r="DL4" t="inlineStr"/>
+      <c r="DL4" t="n">
+        <v>117</v>
+      </c>
       <c r="DM4" t="n">
-        <v>3</v>
-      </c>
-      <c r="DN4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="DN4" t="n">
+        <v>6</v>
+      </c>
       <c r="DO4" t="n">
         <v>2</v>
       </c>
-      <c r="DP4" t="inlineStr"/>
+      <c r="DP4" t="n">
+        <v>214</v>
+      </c>
       <c r="DQ4" t="n">
         <v>3</v>
       </c>
-      <c r="DR4" t="inlineStr"/>
+      <c r="DR4" t="n">
+        <v>47</v>
+      </c>
       <c r="DS4" t="n">
         <v>5</v>
       </c>
@@ -2241,64 +2307,48 @@
         <v>6</v>
       </c>
       <c r="DU4" t="n">
-        <v>2</v>
-      </c>
-      <c r="DV4" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="DV4" t="n">
+        <v>104</v>
+      </c>
       <c r="DW4" t="n">
         <v>3</v>
       </c>
-      <c r="DX4" t="inlineStr"/>
+      <c r="DX4" t="n">
+        <v>72</v>
+      </c>
       <c r="DY4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="DZ4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="EA4" t="n">
-        <v>3</v>
-      </c>
-      <c r="EB4" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="EB4" t="n">
+        <v>7</v>
+      </c>
       <c r="EC4" t="n">
-        <v>3</v>
-      </c>
-      <c r="ED4" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="ED4" t="n">
+        <v>7</v>
+      </c>
       <c r="EE4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="EF4" t="n">
-        <v>7</v>
+        <v>1.962</v>
       </c>
       <c r="EG4" t="n">
-        <v>7</v>
-      </c>
-      <c r="EH4" t="inlineStr"/>
+        <v>1.917</v>
+      </c>
+      <c r="EH4" t="n">
+        <v>2</v>
+      </c>
       <c r="EI4" t="n">
-        <v>7</v>
-      </c>
-      <c r="EJ4" t="inlineStr"/>
-      <c r="EK4" t="inlineStr"/>
-      <c r="EL4" t="inlineStr"/>
-      <c r="EM4" t="inlineStr"/>
-      <c r="EN4" t="inlineStr"/>
-      <c r="EO4" t="n">
-        <v>7</v>
-      </c>
-      <c r="EP4" t="n">
-        <v>7</v>
-      </c>
-      <c r="EQ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="ER4" t="n">
-        <v>1.962</v>
-      </c>
-      <c r="ES4" t="n">
-        <v>1.917</v>
-      </c>
-      <c r="ET4" t="n">
-        <v>2</v>
-      </c>
-      <c r="EU4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2308,156 +2358,416 @@
           <t>P04</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A (B)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2025-03-21</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>29.09.1941</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Apprenticeship</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Stroke (ischemic)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Heart attack</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>87kg</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>manual wheelchair since a few montha</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>27</v>
+      </c>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr"/>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
-      <c r="AX5" t="inlineStr"/>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>3</v>
+      </c>
+      <c r="S5" t="n">
+        <v>35</v>
+      </c>
+      <c r="T5" t="n">
+        <v>3</v>
+      </c>
+      <c r="U5" t="n">
+        <v>17</v>
+      </c>
+      <c r="V5" t="n">
+        <v>3</v>
+      </c>
+      <c r="W5" t="n">
+        <v>28</v>
+      </c>
+      <c r="X5" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>34</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>20</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>110</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>43</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>94</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>108</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>12</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>9</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>0</v>
+      </c>
       <c r="BA5" t="inlineStr"/>
-      <c r="BB5" t="inlineStr"/>
+      <c r="BB5" t="n">
+        <v>0</v>
+      </c>
       <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
-      <c r="BF5" t="inlineStr"/>
+      <c r="BD5" t="n">
+        <v>5</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>5</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
       <c r="BG5" t="inlineStr"/>
-      <c r="BH5" t="inlineStr"/>
+      <c r="BH5" t="n">
+        <v>0</v>
+      </c>
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="inlineStr"/>
       <c r="BK5" t="inlineStr"/>
-      <c r="BL5" t="inlineStr"/>
+      <c r="BL5" t="n">
+        <v>0</v>
+      </c>
       <c r="BM5" t="inlineStr"/>
-      <c r="BN5" t="inlineStr"/>
+      <c r="BN5" t="n">
+        <v>0</v>
+      </c>
       <c r="BO5" t="inlineStr"/>
       <c r="BP5" t="inlineStr"/>
       <c r="BQ5" t="inlineStr"/>
-      <c r="BR5" t="inlineStr"/>
-      <c r="BS5" t="inlineStr"/>
-      <c r="BT5" t="inlineStr"/>
-      <c r="BU5" t="inlineStr"/>
-      <c r="BV5" t="inlineStr"/>
-      <c r="BW5" t="inlineStr"/>
-      <c r="BX5" t="inlineStr"/>
-      <c r="BY5" t="inlineStr"/>
-      <c r="BZ5" t="inlineStr"/>
-      <c r="CA5" t="inlineStr"/>
-      <c r="CB5" t="inlineStr"/>
-      <c r="CC5" t="inlineStr"/>
-      <c r="CD5" t="inlineStr"/>
-      <c r="CE5" t="inlineStr"/>
-      <c r="CF5" t="inlineStr"/>
-      <c r="CG5" t="inlineStr"/>
-      <c r="CH5" t="inlineStr"/>
-      <c r="CI5" t="inlineStr"/>
-      <c r="CJ5" t="inlineStr"/>
-      <c r="CK5" t="inlineStr"/>
-      <c r="CL5" t="inlineStr"/>
-      <c r="CM5" t="inlineStr"/>
-      <c r="CN5" t="inlineStr"/>
-      <c r="CO5" t="inlineStr"/>
-      <c r="CP5" t="inlineStr"/>
-      <c r="CQ5" t="inlineStr"/>
-      <c r="CR5" t="inlineStr"/>
-      <c r="CS5" t="inlineStr"/>
-      <c r="CT5" t="inlineStr"/>
-      <c r="CU5" t="inlineStr"/>
-      <c r="CV5" t="inlineStr"/>
-      <c r="CW5" t="inlineStr"/>
-      <c r="CX5" t="inlineStr"/>
-      <c r="CY5" t="inlineStr"/>
-      <c r="CZ5" t="inlineStr"/>
-      <c r="DA5" t="inlineStr"/>
-      <c r="DB5" t="inlineStr"/>
-      <c r="DC5" t="inlineStr"/>
-      <c r="DD5" t="inlineStr"/>
-      <c r="DE5" t="inlineStr"/>
-      <c r="DF5" t="inlineStr"/>
-      <c r="DG5" t="inlineStr"/>
-      <c r="DH5" t="inlineStr"/>
-      <c r="DI5" t="inlineStr"/>
-      <c r="DJ5" t="inlineStr"/>
-      <c r="DK5" t="inlineStr"/>
-      <c r="DL5" t="inlineStr"/>
-      <c r="DM5" t="inlineStr"/>
-      <c r="DN5" t="inlineStr"/>
-      <c r="DO5" t="inlineStr"/>
-      <c r="DP5" t="inlineStr"/>
-      <c r="DQ5" t="inlineStr"/>
-      <c r="DR5" t="inlineStr"/>
-      <c r="DS5" t="inlineStr"/>
-      <c r="DT5" t="inlineStr"/>
-      <c r="DU5" t="inlineStr"/>
-      <c r="DV5" t="inlineStr"/>
-      <c r="DW5" t="inlineStr"/>
-      <c r="DX5" t="inlineStr"/>
-      <c r="DY5" t="inlineStr"/>
-      <c r="DZ5" t="inlineStr"/>
-      <c r="EA5" t="inlineStr"/>
-      <c r="EB5" t="inlineStr"/>
-      <c r="EC5" t="inlineStr"/>
-      <c r="ED5" t="inlineStr"/>
-      <c r="EE5" t="inlineStr"/>
-      <c r="EF5" t="inlineStr"/>
-      <c r="EG5" t="inlineStr"/>
-      <c r="EH5" t="inlineStr"/>
-      <c r="EI5" t="inlineStr"/>
-      <c r="EJ5" t="inlineStr"/>
-      <c r="EK5" t="inlineStr"/>
-      <c r="EL5" t="inlineStr"/>
-      <c r="EM5" t="inlineStr"/>
-      <c r="EN5" t="inlineStr"/>
-      <c r="EO5" t="inlineStr"/>
-      <c r="EP5" t="inlineStr"/>
-      <c r="EQ5" t="inlineStr"/>
-      <c r="ER5" t="inlineStr"/>
-      <c r="ES5" t="inlineStr"/>
-      <c r="ET5" t="inlineStr"/>
-      <c r="EU5" t="inlineStr"/>
+      <c r="BR5" t="n">
+        <v>6</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>4</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>4</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>6</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>1.231</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="BZ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB5" t="n">
+        <v>78</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>90</v>
+      </c>
+      <c r="CE5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF5" t="n">
+        <v>25</v>
+      </c>
+      <c r="CG5" t="n">
+        <v>4</v>
+      </c>
+      <c r="CH5" t="n">
+        <v>4</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>37</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CL5" t="n">
+        <v>30</v>
+      </c>
+      <c r="CM5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CN5" t="n">
+        <v>9</v>
+      </c>
+      <c r="CO5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP5" t="n">
+        <v>16</v>
+      </c>
+      <c r="CQ5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CR5" t="n">
+        <v>4</v>
+      </c>
+      <c r="CS5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CT5" t="n">
+        <v>65</v>
+      </c>
+      <c r="CU5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CV5" t="n">
+        <v>20</v>
+      </c>
+      <c r="CW5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CX5" t="n">
+        <v>51</v>
+      </c>
+      <c r="CY5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ5" t="n">
+        <v>187</v>
+      </c>
+      <c r="DA5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB5" t="n">
+        <v>96</v>
+      </c>
+      <c r="DC5" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DE5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF5" t="n">
+        <v>19</v>
+      </c>
+      <c r="DG5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DH5" t="n">
+        <v>17</v>
+      </c>
+      <c r="DI5" t="n">
+        <v>2</v>
+      </c>
+      <c r="DJ5" t="n">
+        <v>150</v>
+      </c>
+      <c r="DK5" t="n">
+        <v>2</v>
+      </c>
+      <c r="DL5" t="n">
+        <v>92</v>
+      </c>
+      <c r="DM5" t="n">
+        <v>5</v>
+      </c>
+      <c r="DN5" t="n">
+        <v>4</v>
+      </c>
+      <c r="DO5" t="n">
+        <v>2</v>
+      </c>
+      <c r="DP5" t="n">
+        <v>120</v>
+      </c>
+      <c r="DQ5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DR5" t="n">
+        <v>48</v>
+      </c>
+      <c r="DS5" t="n">
+        <v>4</v>
+      </c>
+      <c r="DT5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DU5" t="n">
+        <v>2</v>
+      </c>
+      <c r="DV5" t="n">
+        <v>128</v>
+      </c>
+      <c r="DW5" t="n">
+        <v>3</v>
+      </c>
+      <c r="DX5" t="n">
+        <v>48</v>
+      </c>
+      <c r="DY5" t="n">
+        <v>4</v>
+      </c>
+      <c r="DZ5" t="n">
+        <v>4</v>
+      </c>
+      <c r="EA5" t="n">
+        <v>6</v>
+      </c>
+      <c r="EB5" t="n">
+        <v>6</v>
+      </c>
+      <c r="EC5" t="n">
+        <v>4</v>
+      </c>
+      <c r="ED5" t="n">
+        <v>6</v>
+      </c>
+      <c r="EE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF5" t="n">
+        <v>0.731</v>
+      </c>
+      <c r="EG5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="EH5" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="EI5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2465,156 +2775,408 @@
           <t>P05</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-04-04</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>10.08.1948</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Apprenticeship</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Parkinson</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>68kg</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="n">
+        <v>27</v>
+      </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr"/>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
-      <c r="BF6" t="inlineStr"/>
-      <c r="BG6" t="inlineStr"/>
-      <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="inlineStr"/>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="inlineStr"/>
-      <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
-      <c r="BQ6" t="inlineStr"/>
-      <c r="BR6" t="inlineStr"/>
-      <c r="BS6" t="inlineStr"/>
-      <c r="BT6" t="inlineStr"/>
-      <c r="BU6" t="inlineStr"/>
-      <c r="BV6" t="inlineStr"/>
-      <c r="BW6" t="inlineStr"/>
-      <c r="BX6" t="inlineStr"/>
-      <c r="BY6" t="inlineStr"/>
-      <c r="BZ6" t="inlineStr"/>
-      <c r="CA6" t="inlineStr"/>
-      <c r="CB6" t="inlineStr"/>
-      <c r="CC6" t="inlineStr"/>
-      <c r="CD6" t="inlineStr"/>
-      <c r="CE6" t="inlineStr"/>
-      <c r="CF6" t="inlineStr"/>
-      <c r="CG6" t="inlineStr"/>
-      <c r="CH6" t="inlineStr"/>
-      <c r="CI6" t="inlineStr"/>
-      <c r="CJ6" t="inlineStr"/>
-      <c r="CK6" t="inlineStr"/>
-      <c r="CL6" t="inlineStr"/>
-      <c r="CM6" t="inlineStr"/>
-      <c r="CN6" t="inlineStr"/>
-      <c r="CO6" t="inlineStr"/>
-      <c r="CP6" t="inlineStr"/>
-      <c r="CQ6" t="inlineStr"/>
-      <c r="CR6" t="inlineStr"/>
-      <c r="CS6" t="inlineStr"/>
-      <c r="CT6" t="inlineStr"/>
-      <c r="CU6" t="inlineStr"/>
-      <c r="CV6" t="inlineStr"/>
-      <c r="CW6" t="inlineStr"/>
-      <c r="CX6" t="inlineStr"/>
-      <c r="CY6" t="inlineStr"/>
-      <c r="CZ6" t="inlineStr"/>
-      <c r="DA6" t="inlineStr"/>
-      <c r="DB6" t="inlineStr"/>
-      <c r="DC6" t="inlineStr"/>
-      <c r="DD6" t="inlineStr"/>
-      <c r="DE6" t="inlineStr"/>
-      <c r="DF6" t="inlineStr"/>
-      <c r="DG6" t="inlineStr"/>
-      <c r="DH6" t="inlineStr"/>
-      <c r="DI6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" t="n">
+        <v>10</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U6" t="n">
+        <v>50</v>
+      </c>
+      <c r="V6" t="n">
+        <v>3</v>
+      </c>
+      <c r="W6" t="n">
+        <v>85</v>
+      </c>
+      <c r="X6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>36</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>31</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>103</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>38</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>260</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>92</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>16</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>11</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>243</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>71</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>4</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>322</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>47</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>351</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>73</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>4</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>6</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>5</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>4</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>4</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>-0.167</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>10</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>130</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF6" t="n">
+        <v>15</v>
+      </c>
+      <c r="CG6" t="n">
+        <v>5</v>
+      </c>
+      <c r="CH6" t="n">
+        <v>6</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>29</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>27</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>30</v>
+      </c>
+      <c r="CO6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>75</v>
+      </c>
+      <c r="CQ6" t="n">
+        <v>4</v>
+      </c>
+      <c r="CR6" t="n">
+        <v>5</v>
+      </c>
+      <c r="CS6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CT6" t="n">
+        <v>55</v>
+      </c>
+      <c r="CU6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CV6" t="n">
+        <v>16</v>
+      </c>
+      <c r="CW6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CX6" t="n">
+        <v>50</v>
+      </c>
+      <c r="CY6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CZ6" t="n">
+        <v>183</v>
+      </c>
+      <c r="DA6" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB6" t="n">
+        <v>103</v>
+      </c>
+      <c r="DC6" t="n">
+        <v>5</v>
+      </c>
+      <c r="DD6" t="n">
+        <v>4</v>
+      </c>
+      <c r="DE6" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF6" t="n">
+        <v>16</v>
+      </c>
+      <c r="DG6" t="n">
+        <v>3</v>
+      </c>
+      <c r="DH6" t="n">
+        <v>14</v>
+      </c>
+      <c r="DI6" t="n">
+        <v>0</v>
+      </c>
       <c r="DJ6" t="inlineStr"/>
-      <c r="DK6" t="inlineStr"/>
+      <c r="DK6" t="n">
+        <v>0</v>
+      </c>
       <c r="DL6" t="inlineStr"/>
-      <c r="DM6" t="inlineStr"/>
-      <c r="DN6" t="inlineStr"/>
-      <c r="DO6" t="inlineStr"/>
+      <c r="DM6" t="n">
+        <v>5</v>
+      </c>
+      <c r="DN6" t="n">
+        <v>5</v>
+      </c>
+      <c r="DO6" t="n">
+        <v>0</v>
+      </c>
       <c r="DP6" t="inlineStr"/>
-      <c r="DQ6" t="inlineStr"/>
+      <c r="DQ6" t="n">
+        <v>0</v>
+      </c>
       <c r="DR6" t="inlineStr"/>
       <c r="DS6" t="inlineStr"/>
       <c r="DT6" t="inlineStr"/>
-      <c r="DU6" t="inlineStr"/>
+      <c r="DU6" t="n">
+        <v>0</v>
+      </c>
       <c r="DV6" t="inlineStr"/>
-      <c r="DW6" t="inlineStr"/>
+      <c r="DW6" t="n">
+        <v>0</v>
+      </c>
       <c r="DX6" t="inlineStr"/>
       <c r="DY6" t="inlineStr"/>
       <c r="DZ6" t="inlineStr"/>
-      <c r="EA6" t="inlineStr"/>
-      <c r="EB6" t="inlineStr"/>
-      <c r="EC6" t="inlineStr"/>
-      <c r="ED6" t="inlineStr"/>
-      <c r="EE6" t="inlineStr"/>
-      <c r="EF6" t="inlineStr"/>
-      <c r="EG6" t="inlineStr"/>
-      <c r="EH6" t="inlineStr"/>
-      <c r="EI6" t="inlineStr"/>
-      <c r="EJ6" t="inlineStr"/>
-      <c r="EK6" t="inlineStr"/>
-      <c r="EL6" t="inlineStr"/>
-      <c r="EM6" t="inlineStr"/>
-      <c r="EN6" t="inlineStr"/>
-      <c r="EO6" t="inlineStr"/>
-      <c r="EP6" t="inlineStr"/>
-      <c r="EQ6" t="inlineStr"/>
-      <c r="ER6" t="inlineStr"/>
-      <c r="ES6" t="inlineStr"/>
-      <c r="ET6" t="inlineStr"/>
-      <c r="EU6" t="inlineStr"/>
+      <c r="EA6" t="n">
+        <v>6</v>
+      </c>
+      <c r="EB6" t="n">
+        <v>5</v>
+      </c>
+      <c r="EC6" t="n">
+        <v>4</v>
+      </c>
+      <c r="ED6" t="n">
+        <v>5</v>
+      </c>
+      <c r="EE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF6" t="n">
+        <v>-115</v>
+      </c>
+      <c r="EG6" t="n">
+        <v>-0.333</v>
+      </c>
+      <c r="EH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EI6" t="n">
+        <v>0.125</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2622,156 +3184,412 @@
           <t>P06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-03-28</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>14.07.1980</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Apprenticeship</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>85kg</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>manual wheelchair at home since 2 years</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="n">
+        <v>28</v>
+      </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
-      <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
-      <c r="BE7" t="inlineStr"/>
-      <c r="BF7" t="inlineStr"/>
-      <c r="BG7" t="inlineStr"/>
-      <c r="BH7" t="inlineStr"/>
-      <c r="BI7" t="inlineStr"/>
-      <c r="BJ7" t="inlineStr"/>
-      <c r="BK7" t="inlineStr"/>
-      <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="inlineStr"/>
-      <c r="BN7" t="inlineStr"/>
-      <c r="BO7" t="inlineStr"/>
-      <c r="BP7" t="inlineStr"/>
-      <c r="BQ7" t="inlineStr"/>
-      <c r="BR7" t="inlineStr"/>
-      <c r="BS7" t="inlineStr"/>
-      <c r="BT7" t="inlineStr"/>
-      <c r="BU7" t="inlineStr"/>
-      <c r="BV7" t="inlineStr"/>
-      <c r="BW7" t="inlineStr"/>
-      <c r="BX7" t="inlineStr"/>
-      <c r="BY7" t="inlineStr"/>
-      <c r="BZ7" t="inlineStr"/>
-      <c r="CA7" t="inlineStr"/>
-      <c r="CB7" t="inlineStr"/>
-      <c r="CC7" t="inlineStr"/>
-      <c r="CD7" t="inlineStr"/>
-      <c r="CE7" t="inlineStr"/>
-      <c r="CF7" t="inlineStr"/>
-      <c r="CG7" t="inlineStr"/>
-      <c r="CH7" t="inlineStr"/>
-      <c r="CI7" t="inlineStr"/>
-      <c r="CJ7" t="inlineStr"/>
-      <c r="CK7" t="inlineStr"/>
-      <c r="CL7" t="inlineStr"/>
-      <c r="CM7" t="inlineStr"/>
-      <c r="CN7" t="inlineStr"/>
-      <c r="CO7" t="inlineStr"/>
-      <c r="CP7" t="inlineStr"/>
-      <c r="CQ7" t="inlineStr"/>
-      <c r="CR7" t="inlineStr"/>
-      <c r="CS7" t="inlineStr"/>
-      <c r="CT7" t="inlineStr"/>
-      <c r="CU7" t="inlineStr"/>
-      <c r="CV7" t="inlineStr"/>
-      <c r="CW7" t="inlineStr"/>
-      <c r="CX7" t="inlineStr"/>
-      <c r="CY7" t="inlineStr"/>
-      <c r="CZ7" t="inlineStr"/>
-      <c r="DA7" t="inlineStr"/>
-      <c r="DB7" t="inlineStr"/>
-      <c r="DC7" t="inlineStr"/>
-      <c r="DD7" t="inlineStr"/>
-      <c r="DE7" t="inlineStr"/>
-      <c r="DF7" t="inlineStr"/>
-      <c r="DG7" t="inlineStr"/>
-      <c r="DH7" t="inlineStr"/>
-      <c r="DI7" t="inlineStr"/>
+      <c r="R7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S7" t="n">
+        <v>17</v>
+      </c>
+      <c r="T7" t="n">
+        <v>3</v>
+      </c>
+      <c r="U7" t="n">
+        <v>10</v>
+      </c>
+      <c r="V7" t="n">
+        <v>3</v>
+      </c>
+      <c r="W7" t="n">
+        <v>21</v>
+      </c>
+      <c r="X7" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>26</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>23</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>74</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>20</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>184</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>42</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>129</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>12</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>10</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>113</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>90</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>140</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>57</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>155</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>102</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>7</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>2.423</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>43</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>30</v>
+      </c>
+      <c r="CE7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF7" t="n">
+        <v>11</v>
+      </c>
+      <c r="CG7" t="n">
+        <v>7</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>7</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>17</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>19</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>8</v>
+      </c>
+      <c r="CO7" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>22</v>
+      </c>
+      <c r="CQ7" t="n">
+        <v>6</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>7</v>
+      </c>
+      <c r="CS7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CT7" t="n">
+        <v>41</v>
+      </c>
+      <c r="CU7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CV7" t="n">
+        <v>12</v>
+      </c>
+      <c r="CW7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CX7" t="n">
+        <v>89</v>
+      </c>
+      <c r="CY7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CZ7" t="n">
+        <v>67</v>
+      </c>
+      <c r="DA7" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB7" t="n">
+        <v>66</v>
+      </c>
+      <c r="DC7" t="n">
+        <v>7</v>
+      </c>
+      <c r="DD7" t="n">
+        <v>7</v>
+      </c>
+      <c r="DE7" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF7" t="n">
+        <v>10</v>
+      </c>
+      <c r="DG7" t="n">
+        <v>3</v>
+      </c>
+      <c r="DH7" t="n">
+        <v>10</v>
+      </c>
+      <c r="DI7" t="n">
+        <v>0</v>
+      </c>
       <c r="DJ7" t="inlineStr"/>
-      <c r="DK7" t="inlineStr"/>
+      <c r="DK7" t="n">
+        <v>0</v>
+      </c>
       <c r="DL7" t="inlineStr"/>
-      <c r="DM7" t="inlineStr"/>
-      <c r="DN7" t="inlineStr"/>
-      <c r="DO7" t="inlineStr"/>
+      <c r="DM7" t="n">
+        <v>7</v>
+      </c>
+      <c r="DN7" t="n">
+        <v>7</v>
+      </c>
+      <c r="DO7" t="n">
+        <v>0</v>
+      </c>
       <c r="DP7" t="inlineStr"/>
-      <c r="DQ7" t="inlineStr"/>
+      <c r="DQ7" t="n">
+        <v>0</v>
+      </c>
       <c r="DR7" t="inlineStr"/>
       <c r="DS7" t="inlineStr"/>
       <c r="DT7" t="inlineStr"/>
-      <c r="DU7" t="inlineStr"/>
+      <c r="DU7" t="n">
+        <v>0</v>
+      </c>
       <c r="DV7" t="inlineStr"/>
-      <c r="DW7" t="inlineStr"/>
+      <c r="DW7" t="n">
+        <v>0</v>
+      </c>
       <c r="DX7" t="inlineStr"/>
       <c r="DY7" t="inlineStr"/>
       <c r="DZ7" t="inlineStr"/>
-      <c r="EA7" t="inlineStr"/>
-      <c r="EB7" t="inlineStr"/>
-      <c r="EC7" t="inlineStr"/>
-      <c r="ED7" t="inlineStr"/>
-      <c r="EE7" t="inlineStr"/>
-      <c r="EF7" t="inlineStr"/>
-      <c r="EG7" t="inlineStr"/>
-      <c r="EH7" t="inlineStr"/>
-      <c r="EI7" t="inlineStr"/>
-      <c r="EJ7" t="inlineStr"/>
-      <c r="EK7" t="inlineStr"/>
-      <c r="EL7" t="inlineStr"/>
-      <c r="EM7" t="inlineStr"/>
-      <c r="EN7" t="inlineStr"/>
-      <c r="EO7" t="inlineStr"/>
-      <c r="EP7" t="inlineStr"/>
-      <c r="EQ7" t="inlineStr"/>
-      <c r="ER7" t="inlineStr"/>
-      <c r="ES7" t="inlineStr"/>
-      <c r="ET7" t="inlineStr"/>
-      <c r="EU7" t="inlineStr"/>
+      <c r="EA7" t="n">
+        <v>6</v>
+      </c>
+      <c r="EB7" t="n">
+        <v>6</v>
+      </c>
+      <c r="EC7" t="n">
+        <v>7</v>
+      </c>
+      <c r="ED7" t="n">
+        <v>7</v>
+      </c>
+      <c r="EE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF7" t="n">
+        <v>2.846</v>
+      </c>
+      <c r="EG7" t="n">
+        <v>2.833</v>
+      </c>
+      <c r="EH7" t="n">
+        <v>3</v>
+      </c>
+      <c r="EI7" t="n">
+        <v>2.75</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2779,156 +3597,420 @@
           <t>P07</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-04-04</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>13.09.1959</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Apprenticeship</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Stroke</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>46kg</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2 (left), 0(right)</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>magic Mobility since 2 years extreme x8</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>28</v>
+      </c>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
-      <c r="BF8" t="inlineStr"/>
-      <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
-      <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="inlineStr"/>
-      <c r="BK8" t="inlineStr"/>
-      <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="inlineStr"/>
-      <c r="BN8" t="inlineStr"/>
-      <c r="BO8" t="inlineStr"/>
-      <c r="BP8" t="inlineStr"/>
-      <c r="BQ8" t="inlineStr"/>
-      <c r="BR8" t="inlineStr"/>
-      <c r="BS8" t="inlineStr"/>
-      <c r="BT8" t="inlineStr"/>
-      <c r="BU8" t="inlineStr"/>
-      <c r="BV8" t="inlineStr"/>
-      <c r="BW8" t="inlineStr"/>
-      <c r="BX8" t="inlineStr"/>
-      <c r="BY8" t="inlineStr"/>
-      <c r="BZ8" t="inlineStr"/>
-      <c r="CA8" t="inlineStr"/>
-      <c r="CB8" t="inlineStr"/>
-      <c r="CC8" t="inlineStr"/>
-      <c r="CD8" t="inlineStr"/>
-      <c r="CE8" t="inlineStr"/>
-      <c r="CF8" t="inlineStr"/>
-      <c r="CG8" t="inlineStr"/>
-      <c r="CH8" t="inlineStr"/>
-      <c r="CI8" t="inlineStr"/>
-      <c r="CJ8" t="inlineStr"/>
-      <c r="CK8" t="inlineStr"/>
-      <c r="CL8" t="inlineStr"/>
-      <c r="CM8" t="inlineStr"/>
-      <c r="CN8" t="inlineStr"/>
-      <c r="CO8" t="inlineStr"/>
-      <c r="CP8" t="inlineStr"/>
-      <c r="CQ8" t="inlineStr"/>
-      <c r="CR8" t="inlineStr"/>
-      <c r="CS8" t="inlineStr"/>
-      <c r="CT8" t="inlineStr"/>
-      <c r="CU8" t="inlineStr"/>
-      <c r="CV8" t="inlineStr"/>
-      <c r="CW8" t="inlineStr"/>
-      <c r="CX8" t="inlineStr"/>
-      <c r="CY8" t="inlineStr"/>
-      <c r="CZ8" t="inlineStr"/>
-      <c r="DA8" t="inlineStr"/>
-      <c r="DB8" t="inlineStr"/>
-      <c r="DC8" t="inlineStr"/>
-      <c r="DD8" t="inlineStr"/>
-      <c r="DE8" t="inlineStr"/>
-      <c r="DF8" t="inlineStr"/>
-      <c r="DG8" t="inlineStr"/>
-      <c r="DH8" t="inlineStr"/>
-      <c r="DI8" t="inlineStr"/>
+      <c r="R8" t="n">
+        <v>3</v>
+      </c>
+      <c r="S8" t="n">
+        <v>23</v>
+      </c>
+      <c r="T8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" t="n">
+        <v>164</v>
+      </c>
+      <c r="V8" t="n">
+        <v>3</v>
+      </c>
+      <c r="W8" t="n">
+        <v>53</v>
+      </c>
+      <c r="X8" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>41</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>13</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>20</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>6</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>6</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>242</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>228</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>700</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>255</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>154</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>15</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>12</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>175</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>148</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>6</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>5</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>180</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>64</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>5</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>138</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>111</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>6</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>6</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>6</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>6</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>5</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>7</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>2.192</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>1.833</v>
+      </c>
+      <c r="BZ8" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB8" t="n">
+        <v>14</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>32</v>
+      </c>
+      <c r="CE8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CF8" t="n">
+        <v>13</v>
+      </c>
+      <c r="CG8" t="n">
+        <v>7</v>
+      </c>
+      <c r="CH8" t="n">
+        <v>7</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>16</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>12</v>
+      </c>
+      <c r="CM8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CN8" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO8" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP8" t="n">
+        <v>31</v>
+      </c>
+      <c r="CQ8" t="n">
+        <v>5</v>
+      </c>
+      <c r="CR8" t="n">
+        <v>6</v>
+      </c>
+      <c r="CS8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CT8" t="n">
+        <v>48</v>
+      </c>
+      <c r="CU8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CV8" t="n">
+        <v>23</v>
+      </c>
+      <c r="CW8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CX8" t="n">
+        <v>102</v>
+      </c>
+      <c r="CY8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CZ8" t="n">
+        <v>33</v>
+      </c>
+      <c r="DA8" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB8" t="n">
+        <v>95</v>
+      </c>
+      <c r="DC8" t="n">
+        <v>6</v>
+      </c>
+      <c r="DD8" t="n">
+        <v>5</v>
+      </c>
+      <c r="DE8" t="n">
+        <v>3</v>
+      </c>
+      <c r="DF8" t="n">
+        <v>14</v>
+      </c>
+      <c r="DG8" t="n">
+        <v>3</v>
+      </c>
+      <c r="DH8" t="n">
+        <v>12</v>
+      </c>
+      <c r="DI8" t="n">
+        <v>0</v>
+      </c>
       <c r="DJ8" t="inlineStr"/>
-      <c r="DK8" t="inlineStr"/>
+      <c r="DK8" t="n">
+        <v>0</v>
+      </c>
       <c r="DL8" t="inlineStr"/>
-      <c r="DM8" t="inlineStr"/>
-      <c r="DN8" t="inlineStr"/>
-      <c r="DO8" t="inlineStr"/>
+      <c r="DM8" t="n">
+        <v>7</v>
+      </c>
+      <c r="DN8" t="n">
+        <v>7</v>
+      </c>
+      <c r="DO8" t="n">
+        <v>0</v>
+      </c>
       <c r="DP8" t="inlineStr"/>
-      <c r="DQ8" t="inlineStr"/>
+      <c r="DQ8" t="n">
+        <v>0</v>
+      </c>
       <c r="DR8" t="inlineStr"/>
       <c r="DS8" t="inlineStr"/>
       <c r="DT8" t="inlineStr"/>
-      <c r="DU8" t="inlineStr"/>
+      <c r="DU8" t="n">
+        <v>0</v>
+      </c>
       <c r="DV8" t="inlineStr"/>
-      <c r="DW8" t="inlineStr"/>
+      <c r="DW8" t="n">
+        <v>0</v>
+      </c>
       <c r="DX8" t="inlineStr"/>
       <c r="DY8" t="inlineStr"/>
       <c r="DZ8" t="inlineStr"/>
-      <c r="EA8" t="inlineStr"/>
-      <c r="EB8" t="inlineStr"/>
-      <c r="EC8" t="inlineStr"/>
-      <c r="ED8" t="inlineStr"/>
-      <c r="EE8" t="inlineStr"/>
-      <c r="EF8" t="inlineStr"/>
-      <c r="EG8" t="inlineStr"/>
-      <c r="EH8" t="inlineStr"/>
-      <c r="EI8" t="inlineStr"/>
-      <c r="EJ8" t="inlineStr"/>
-      <c r="EK8" t="inlineStr"/>
-      <c r="EL8" t="inlineStr"/>
-      <c r="EM8" t="inlineStr"/>
-      <c r="EN8" t="inlineStr"/>
-      <c r="EO8" t="inlineStr"/>
-      <c r="EP8" t="inlineStr"/>
-      <c r="EQ8" t="inlineStr"/>
-      <c r="ER8" t="inlineStr"/>
-      <c r="ES8" t="inlineStr"/>
-      <c r="ET8" t="inlineStr"/>
-      <c r="EU8" t="inlineStr"/>
+      <c r="EA8" t="n">
+        <v>7</v>
+      </c>
+      <c r="EB8" t="n">
+        <v>7</v>
+      </c>
+      <c r="EC8" t="n">
+        <v>6</v>
+      </c>
+      <c r="ED8" t="n">
+        <v>6</v>
+      </c>
+      <c r="EE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF8" t="n">
+        <v>1.808</v>
+      </c>
+      <c r="EG8" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="EH8" t="n">
+        <v>1.833</v>
+      </c>
+      <c r="EI8" t="n">
+        <v>1.875</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2936,7 +4018,11 @@
           <t>P08</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
@@ -3074,18 +4160,6 @@
       <c r="EG9" t="inlineStr"/>
       <c r="EH9" t="inlineStr"/>
       <c r="EI9" t="inlineStr"/>
-      <c r="EJ9" t="inlineStr"/>
-      <c r="EK9" t="inlineStr"/>
-      <c r="EL9" t="inlineStr"/>
-      <c r="EM9" t="inlineStr"/>
-      <c r="EN9" t="inlineStr"/>
-      <c r="EO9" t="inlineStr"/>
-      <c r="EP9" t="inlineStr"/>
-      <c r="EQ9" t="inlineStr"/>
-      <c r="ER9" t="inlineStr"/>
-      <c r="ES9" t="inlineStr"/>
-      <c r="ET9" t="inlineStr"/>
-      <c r="EU9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3231,18 +4305,6 @@
       <c r="EG10" t="inlineStr"/>
       <c r="EH10" t="inlineStr"/>
       <c r="EI10" t="inlineStr"/>
-      <c r="EJ10" t="inlineStr"/>
-      <c r="EK10" t="inlineStr"/>
-      <c r="EL10" t="inlineStr"/>
-      <c r="EM10" t="inlineStr"/>
-      <c r="EN10" t="inlineStr"/>
-      <c r="EO10" t="inlineStr"/>
-      <c r="EP10" t="inlineStr"/>
-      <c r="EQ10" t="inlineStr"/>
-      <c r="ER10" t="inlineStr"/>
-      <c r="ES10" t="inlineStr"/>
-      <c r="ET10" t="inlineStr"/>
-      <c r="EU10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3388,18 +4450,6 @@
       <c r="EG11" t="inlineStr"/>
       <c r="EH11" t="inlineStr"/>
       <c r="EI11" t="inlineStr"/>
-      <c r="EJ11" t="inlineStr"/>
-      <c r="EK11" t="inlineStr"/>
-      <c r="EL11" t="inlineStr"/>
-      <c r="EM11" t="inlineStr"/>
-      <c r="EN11" t="inlineStr"/>
-      <c r="EO11" t="inlineStr"/>
-      <c r="EP11" t="inlineStr"/>
-      <c r="EQ11" t="inlineStr"/>
-      <c r="ER11" t="inlineStr"/>
-      <c r="ES11" t="inlineStr"/>
-      <c r="ET11" t="inlineStr"/>
-      <c r="EU11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3545,18 +4595,6 @@
       <c r="EG12" t="inlineStr"/>
       <c r="EH12" t="inlineStr"/>
       <c r="EI12" t="inlineStr"/>
-      <c r="EJ12" t="inlineStr"/>
-      <c r="EK12" t="inlineStr"/>
-      <c r="EL12" t="inlineStr"/>
-      <c r="EM12" t="inlineStr"/>
-      <c r="EN12" t="inlineStr"/>
-      <c r="EO12" t="inlineStr"/>
-      <c r="EP12" t="inlineStr"/>
-      <c r="EQ12" t="inlineStr"/>
-      <c r="ER12" t="inlineStr"/>
-      <c r="ES12" t="inlineStr"/>
-      <c r="ET12" t="inlineStr"/>
-      <c r="EU12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3702,18 +4740,6 @@
       <c r="EG13" t="inlineStr"/>
       <c r="EH13" t="inlineStr"/>
       <c r="EI13" t="inlineStr"/>
-      <c r="EJ13" t="inlineStr"/>
-      <c r="EK13" t="inlineStr"/>
-      <c r="EL13" t="inlineStr"/>
-      <c r="EM13" t="inlineStr"/>
-      <c r="EN13" t="inlineStr"/>
-      <c r="EO13" t="inlineStr"/>
-      <c r="EP13" t="inlineStr"/>
-      <c r="EQ13" t="inlineStr"/>
-      <c r="ER13" t="inlineStr"/>
-      <c r="ES13" t="inlineStr"/>
-      <c r="ET13" t="inlineStr"/>
-      <c r="EU13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3859,18 +4885,6 @@
       <c r="EG14" t="inlineStr"/>
       <c r="EH14" t="inlineStr"/>
       <c r="EI14" t="inlineStr"/>
-      <c r="EJ14" t="inlineStr"/>
-      <c r="EK14" t="inlineStr"/>
-      <c r="EL14" t="inlineStr"/>
-      <c r="EM14" t="inlineStr"/>
-      <c r="EN14" t="inlineStr"/>
-      <c r="EO14" t="inlineStr"/>
-      <c r="EP14" t="inlineStr"/>
-      <c r="EQ14" t="inlineStr"/>
-      <c r="ER14" t="inlineStr"/>
-      <c r="ES14" t="inlineStr"/>
-      <c r="ET14" t="inlineStr"/>
-      <c r="EU14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4016,18 +5030,6 @@
       <c r="EG15" t="inlineStr"/>
       <c r="EH15" t="inlineStr"/>
       <c r="EI15" t="inlineStr"/>
-      <c r="EJ15" t="inlineStr"/>
-      <c r="EK15" t="inlineStr"/>
-      <c r="EL15" t="inlineStr"/>
-      <c r="EM15" t="inlineStr"/>
-      <c r="EN15" t="inlineStr"/>
-      <c r="EO15" t="inlineStr"/>
-      <c r="EP15" t="inlineStr"/>
-      <c r="EQ15" t="inlineStr"/>
-      <c r="ER15" t="inlineStr"/>
-      <c r="ES15" t="inlineStr"/>
-      <c r="ET15" t="inlineStr"/>
-      <c r="EU15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4173,18 +5175,6 @@
       <c r="EG16" t="inlineStr"/>
       <c r="EH16" t="inlineStr"/>
       <c r="EI16" t="inlineStr"/>
-      <c r="EJ16" t="inlineStr"/>
-      <c r="EK16" t="inlineStr"/>
-      <c r="EL16" t="inlineStr"/>
-      <c r="EM16" t="inlineStr"/>
-      <c r="EN16" t="inlineStr"/>
-      <c r="EO16" t="inlineStr"/>
-      <c r="EP16" t="inlineStr"/>
-      <c r="EQ16" t="inlineStr"/>
-      <c r="ER16" t="inlineStr"/>
-      <c r="ES16" t="inlineStr"/>
-      <c r="ET16" t="inlineStr"/>
-      <c r="EU16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4330,18 +5320,6 @@
       <c r="EG17" t="inlineStr"/>
       <c r="EH17" t="inlineStr"/>
       <c r="EI17" t="inlineStr"/>
-      <c r="EJ17" t="inlineStr"/>
-      <c r="EK17" t="inlineStr"/>
-      <c r="EL17" t="inlineStr"/>
-      <c r="EM17" t="inlineStr"/>
-      <c r="EN17" t="inlineStr"/>
-      <c r="EO17" t="inlineStr"/>
-      <c r="EP17" t="inlineStr"/>
-      <c r="EQ17" t="inlineStr"/>
-      <c r="ER17" t="inlineStr"/>
-      <c r="ES17" t="inlineStr"/>
-      <c r="ET17" t="inlineStr"/>
-      <c r="EU17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4487,18 +5465,6 @@
       <c r="EG18" t="inlineStr"/>
       <c r="EH18" t="inlineStr"/>
       <c r="EI18" t="inlineStr"/>
-      <c r="EJ18" t="inlineStr"/>
-      <c r="EK18" t="inlineStr"/>
-      <c r="EL18" t="inlineStr"/>
-      <c r="EM18" t="inlineStr"/>
-      <c r="EN18" t="inlineStr"/>
-      <c r="EO18" t="inlineStr"/>
-      <c r="EP18" t="inlineStr"/>
-      <c r="EQ18" t="inlineStr"/>
-      <c r="ER18" t="inlineStr"/>
-      <c r="ES18" t="inlineStr"/>
-      <c r="ET18" t="inlineStr"/>
-      <c r="EU18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4644,18 +5610,6 @@
       <c r="EG19" t="inlineStr"/>
       <c r="EH19" t="inlineStr"/>
       <c r="EI19" t="inlineStr"/>
-      <c r="EJ19" t="inlineStr"/>
-      <c r="EK19" t="inlineStr"/>
-      <c r="EL19" t="inlineStr"/>
-      <c r="EM19" t="inlineStr"/>
-      <c r="EN19" t="inlineStr"/>
-      <c r="EO19" t="inlineStr"/>
-      <c r="EP19" t="inlineStr"/>
-      <c r="EQ19" t="inlineStr"/>
-      <c r="ER19" t="inlineStr"/>
-      <c r="ES19" t="inlineStr"/>
-      <c r="ET19" t="inlineStr"/>
-      <c r="EU19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4801,18 +5755,6 @@
       <c r="EG20" t="inlineStr"/>
       <c r="EH20" t="inlineStr"/>
       <c r="EI20" t="inlineStr"/>
-      <c r="EJ20" t="inlineStr"/>
-      <c r="EK20" t="inlineStr"/>
-      <c r="EL20" t="inlineStr"/>
-      <c r="EM20" t="inlineStr"/>
-      <c r="EN20" t="inlineStr"/>
-      <c r="EO20" t="inlineStr"/>
-      <c r="EP20" t="inlineStr"/>
-      <c r="EQ20" t="inlineStr"/>
-      <c r="ER20" t="inlineStr"/>
-      <c r="ES20" t="inlineStr"/>
-      <c r="ET20" t="inlineStr"/>
-      <c r="EU20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4958,18 +5900,6 @@
       <c r="EG21" t="inlineStr"/>
       <c r="EH21" t="inlineStr"/>
       <c r="EI21" t="inlineStr"/>
-      <c r="EJ21" t="inlineStr"/>
-      <c r="EK21" t="inlineStr"/>
-      <c r="EL21" t="inlineStr"/>
-      <c r="EM21" t="inlineStr"/>
-      <c r="EN21" t="inlineStr"/>
-      <c r="EO21" t="inlineStr"/>
-      <c r="EP21" t="inlineStr"/>
-      <c r="EQ21" t="inlineStr"/>
-      <c r="ER21" t="inlineStr"/>
-      <c r="ES21" t="inlineStr"/>
-      <c r="ET21" t="inlineStr"/>
-      <c r="EU21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5115,18 +6045,6 @@
       <c r="EG22" t="inlineStr"/>
       <c r="EH22" t="inlineStr"/>
       <c r="EI22" t="inlineStr"/>
-      <c r="EJ22" t="inlineStr"/>
-      <c r="EK22" t="inlineStr"/>
-      <c r="EL22" t="inlineStr"/>
-      <c r="EM22" t="inlineStr"/>
-      <c r="EN22" t="inlineStr"/>
-      <c r="EO22" t="inlineStr"/>
-      <c r="EP22" t="inlineStr"/>
-      <c r="EQ22" t="inlineStr"/>
-      <c r="ER22" t="inlineStr"/>
-      <c r="ES22" t="inlineStr"/>
-      <c r="ET22" t="inlineStr"/>
-      <c r="EU22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5272,18 +6190,6 @@
       <c r="EG23" t="inlineStr"/>
       <c r="EH23" t="inlineStr"/>
       <c r="EI23" t="inlineStr"/>
-      <c r="EJ23" t="inlineStr"/>
-      <c r="EK23" t="inlineStr"/>
-      <c r="EL23" t="inlineStr"/>
-      <c r="EM23" t="inlineStr"/>
-      <c r="EN23" t="inlineStr"/>
-      <c r="EO23" t="inlineStr"/>
-      <c r="EP23" t="inlineStr"/>
-      <c r="EQ23" t="inlineStr"/>
-      <c r="ER23" t="inlineStr"/>
-      <c r="ES23" t="inlineStr"/>
-      <c r="ET23" t="inlineStr"/>
-      <c r="EU23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>